<commit_message>
B6: envelope at the engine plan, 900% wall rule, live values, test budgets
Envelope $619/day (engine after-audit spend) for 09-24..09-28; base carries the
raise past the 900% modifier wall; rows priced from live 22 Sep values; third
in-focus campaign with no bid added; out-of-focus tests on budgets sized to ~15
TOS clicks; claims tightened (price buys share, tuning explains part of the drop,
campaign-level CVR for King/Queen/Full); run-action counts reconciled.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvXHKtbYmE3ru99HYV2muV
</commit_message>
<xml_diff>
--- a/docs/DBS6_Corrections_by_Situation_20260921-f066a8f0.xlsx
+++ b/docs/DBS6_Corrections_by_Situation_20260921-f066a8f0.xlsx
@@ -1530,7 +1530,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Push TOS +20% (no click requirement on file → +20% (a stated departure: the logic document would hold at the ceiling)): $7.93 → $9.52; modifier 543%; daily read to 09-28</t>
+          <t>Push TOS +20% (no click requirement on file → +20% (a stated departure: the logic document would hold at the ceiling)): $10.32 → $12.38; modifier 736%; daily read to 09-28</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2593,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Push TOS +20% (no click requirement on file → +20% (a stated departure: the logic document would hold at the ceiling)): $6.42 → $7.70; modifier 316%; re-point the ad to the serving child; daily read to 09-28</t>
+          <t>Push TOS +20% (no click requirement on file → +20% (a stated departure: the logic document would hold at the ceiling)): $8.34 → $10.01; modifier 441%; re-point the ad to the serving child; daily read to 09-28</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>Push TOS +20% (no click requirement on file → +20% (a stated departure: the logic document would hold at the ceiling)): $7.93 → $9.52; modifier 543%; daily read to 09-28</t>
+          <t>Push TOS +20% (no click requirement on file → +20% (a stated departure: the logic document would hold at the ceiling)): $10.32 → $12.38; modifier 736%; daily read to 09-28</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>Restore pre-cut prices, then push TOS +30% (1% of required top-of-search clicks delivered → +30%): $4.80 → $6.24; base held; modifier would pass the 900% wall — base lifted as a stated trade: base $0.50 → $0.62; modifier 900%; daily read to 09-28</t>
+          <t>Restore pre-cut prices, then push TOS +30% (1% of required top-of-search clicks delivered → +30%): $4.80 → $6.24; base held; the modifier would pass the 900% wall, so the base carries the raise (0.50 → 0.62) at 900% — watch product-page share the next day: base $0.50 → $0.62; modifier 900%; daily read to 09-28</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>Out of focus but converts (24% at top of search vs bar 10.5%): test TOS +10% $3.46 → $3.80 to 10-07; restore the pre-cut base first</t>
+          <t>Out of focus but converts (24% at top of search vs bar 10.5%): test TOS +10% $3.46 → $3.80 to 10-07; budget $5.00/day; restore the pre-cut base first</t>
         </is>
       </c>
     </row>
@@ -4195,7 +4195,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>Out of focus but converts (13% at top of search vs bar 10.5%): test TOS +10% $3.74 → $4.12 to 10-07</t>
+          <t>Out of focus but converts (13% at top of search vs bar 10.5%): test TOS +10% $3.74 → $4.12 to 10-07; budget $5.00/day</t>
         </is>
       </c>
     </row>
@@ -4262,7 +4262,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>Out of focus but converts (15% at top of search vs bar 5.5%): test TOS +10% $3.16 → $3.48 to 10-07; advertise BAMBOO-QUEEN-OLIVE-6PCS; restore the pre-cut base first</t>
+          <t>Out of focus but converts (15% at top of search vs bar 5.5%): test TOS +10% $3.16 → $3.48 to 10-07; budget $5.00/day; advertise BAMBOO-QUEEN-OLIVE-6PCS; restore the pre-cut base first</t>
         </is>
       </c>
     </row>
@@ -4329,7 +4329,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>Out of focus but converts (29% at top of search vs bar 13.3%): test TOS +10% $5.17 → $5.69 to 10-07; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
+          <t>Out of focus but converts (29% at top of search vs bar 13.3%): test TOS +10% $5.17 → $5.69 to 10-07; budget $6.09/day; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
         </is>
       </c>
     </row>
@@ -4396,7 +4396,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>Out of focus but converts (21% at top of search vs bar 12.6%): test TOS +10% $4.56 → $5.01 to 10-07; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
+          <t>Out of focus but converts (21% at top of search vs bar 12.6%): test TOS +10% $4.56 → $5.01 to 10-07; budget $5.37/day; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
         </is>
       </c>
     </row>
@@ -4527,7 +4527,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>Out of focus but converts (11% at top of search vs bar 10.9%): test TOS +10% $1.35 → $1.49 to 10-07</t>
+          <t>Out of focus but converts (11% at top of search vs bar 10.9%): test TOS +10% $1.35 → $1.49 to 10-07; budget $5.00/day</t>
         </is>
       </c>
     </row>
@@ -4594,7 +4594,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>Out of focus but converts (33% at top of search vs bar 6.4%): test TOS +10% $6.36 → $7.00 to 10-07; advertise BAMBOO-QUEEN-OLIVE-6PCS; restore the pre-cut base first</t>
+          <t>Out of focus but converts (33% at top of search vs bar 6.4%): test TOS +10% $6.36 → $7.00 to 10-07; budget $7.50/day; advertise BAMBOO-QUEEN-OLIVE-6PCS; restore the pre-cut base first</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>Out of focus but converts (21% at top of search vs bar 13.3%): test TOS +10% $5.71 → $6.28 to 10-07; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
+          <t>Out of focus but converts (21% at top of search vs bar 13.3%): test TOS +10% $5.71 → $6.28 to 10-07; budget $6.73/day; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
         </is>
       </c>
     </row>
@@ -4728,7 +4728,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Out of focus but converts (19% at top of search vs bar 12.4%): test TOS +10% $4.81 → $5.29 to 10-07; advertise BAMBOO-FULL-CREME-6PCS</t>
+          <t>Out of focus but converts (19% at top of search vs bar 12.4%): test TOS +10% $4.81 → $5.29 to 10-07; budget $5.67/day; advertise BAMBOO-FULL-CREME-6PCS</t>
         </is>
       </c>
     </row>
@@ -4795,7 +4795,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>Out of focus but converts (11% at top of search vs bar 10.5%): test TOS +10% $5.72 → $6.29 to 10-07</t>
+          <t>Out of focus but converts (11% at top of search vs bar 10.5%): test TOS +10% $5.72 → $6.29 to 10-07; budget $6.74/day</t>
         </is>
       </c>
     </row>
@@ -4862,7 +4862,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>Out of focus but converts (17% at top of search vs bar 10.5%): test TOS +10% $5.43 → $5.98 to 10-07; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
+          <t>Out of focus but converts (17% at top of search vs bar 10.5%): test TOS +10% $5.43 → $5.98 to 10-07; budget $6.40/day; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
         </is>
       </c>
     </row>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>Out of focus but converts (12% at top of search vs bar 10.5%): test TOS +10% $5.03 → $5.54 to 10-07; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
+          <t>Out of focus but converts (12% at top of search vs bar 10.5%): test TOS +10% $5.03 → $5.54 to 10-07; budget $5.93/day; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
         </is>
       </c>
     </row>
@@ -4996,7 +4996,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>Out of focus but converts (22% at top of search vs bar 10.5%): test TOS +10% $4.29 → $4.72 to 10-07</t>
+          <t>Out of focus but converts (22% at top of search vs bar 10.5%): test TOS +10% $4.29 → $4.72 to 10-07; budget $5.06/day</t>
         </is>
       </c>
     </row>
@@ -5063,7 +5063,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>Out of focus but converts (18% at top of search vs bar 10.5%): test TOS +10% $3.34 → $3.68 to 10-07; restore the pre-cut base first</t>
+          <t>Out of focus but converts (18% at top of search vs bar 10.5%): test TOS +10% $3.34 → $3.68 to 10-07; budget $5.00/day; restore the pre-cut base first</t>
         </is>
       </c>
     </row>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>Out of focus but converts (21% at top of search vs bar 10.5%): test TOS +10% $3.84 → $4.23 to 10-07; advertise BAMBOO-QUEEN-OLIVE-6PCS; restore the pre-cut base first</t>
+          <t>Out of focus but converts (21% at top of search vs bar 10.5%): test TOS +10% $3.84 → $4.23 to 10-07; budget $5.00/day; advertise BAMBOO-QUEEN-OLIVE-6PCS; restore the pre-cut base first</t>
         </is>
       </c>
     </row>
@@ -5197,7 +5197,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>Out of focus but converts (42% at top of search vs bar 20.1%): test TOS +10% $3.54 → $3.89 to 10-07</t>
+          <t>Out of focus but converts (42% at top of search vs bar 20.1%): test TOS +10% $3.54 → $3.89 to 10-07; budget $5.00/day</t>
         </is>
       </c>
     </row>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>Out of focus but converts (27% at top of search vs bar 13.3%): test TOS +10% $2.01 → $2.22 to 10-07; advertise BAMBOO-QUEEN-OLIVE-6PCS; restore the pre-cut base first</t>
+          <t>Out of focus but converts (27% at top of search vs bar 13.3%): test TOS +10% $2.01 → $2.22 to 10-07; budget $5.00/day; advertise BAMBOO-QUEEN-OLIVE-6PCS; restore the pre-cut base first</t>
         </is>
       </c>
     </row>
@@ -5331,7 +5331,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>Out of focus but converts (26% at top of search vs bar 5.8%): test TOS +10% $4.24 → $4.67 to 10-07</t>
+          <t>Out of focus but converts (26% at top of search vs bar 5.8%): test TOS +10% $4.24 → $4.67 to 10-07; budget $5.00/day</t>
         </is>
       </c>
     </row>
@@ -5398,7 +5398,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>Out of focus but converts (16% at top of search vs bar 13.3%): test TOS +10% $7.30 → $8.03 to 10-07; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
+          <t>Out of focus but converts (16% at top of search vs bar 13.3%): test TOS +10% $7.30 → $8.03 to 10-07; budget $8.60/day; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
         </is>
       </c>
     </row>
@@ -5465,7 +5465,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>Out of focus but converts (13% at top of search vs bar 13.3%): test TOS +10% $6.06 → $6.67 to 10-07; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
+          <t>Out of focus but converts (13% at top of search vs bar 13.3%): test TOS +10% $6.06 → $6.67 to 10-07; budget $7.15/day; advertise BAMBOO-QUEEN-OLIVE-6PCS</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>Out of focus but converts (28% at top of search vs bar 13.3%): test TOS +10% $6.07 → $6.67 to 10-07; advertise BAMBOO-QUEEN-OLIVE-6PCS; restore the pre-cut base first</t>
+          <t>Out of focus but converts (28% at top of search vs bar 13.3%): test TOS +10% $6.07 → $6.67 to 10-07; budget $7.15/day; advertise BAMBOO-QUEEN-OLIVE-6PCS; restore the pre-cut base first</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>Out of focus but converts (27% at top of search vs bar 16.0%): test TOS +10% $5.04 → $5.54 to 10-07; restore the pre-cut base first</t>
+          <t>Out of focus but converts (27% at top of search vs bar 16.0%): test TOS +10% $5.04 → $5.54 to 10-07; budget $5.94/day; restore the pre-cut base first</t>
         </is>
       </c>
     </row>

</xml_diff>